<commit_message>
added nicole kilo WCH 2025
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SamB\OneDrive - SportNZGroup\Desktop\Scripts\Para Tracker\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sportnzgroup-my.sharepoint.com/personal/sam_bremer_hpsnz_org_nz/Documents/Desktop/Scripts/Para Tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6954CE-EC5B-43AB-B923-0C939D68B3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{1C6954CE-EC5B-43AB-B923-0C939D68B3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C92BAA3A-AE7F-4258-83EE-FFFFFDE73DC4}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="10800" windowWidth="19420" windowHeight="10300" xr2:uid="{0366F0DF-8659-49CC-A902-2A4788A5E28D}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="41">
   <si>
     <t>Name</t>
   </si>
@@ -548,7 +548,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24732CBF-5850-4CE8-9E62-B42B0032864B}">
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="13.53125" bestFit="1" customWidth="1"/>
@@ -2182,42 +2182,42 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B57" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C57" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D57" t="s">
         <v>22</v>
       </c>
       <c r="E57" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F57" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G57" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="H57" s="1">
-        <v>46065</v>
+        <v>45946</v>
       </c>
       <c r="I57" s="2">
-        <v>8.4380787037037041E-4</v>
+        <v>8.4773148148148143E-4</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B58" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C58" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D58" t="s">
         <v>22</v>
@@ -2226,16 +2226,16 @@
         <v>12</v>
       </c>
       <c r="F58" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G58" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="H58" s="1">
-        <v>45844</v>
+        <v>45946</v>
       </c>
       <c r="I58" s="2">
-        <v>8.5418981481481468E-4</v>
+        <v>8.5207175925925923E-4</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.45">
@@ -2252,19 +2252,19 @@
         <v>22</v>
       </c>
       <c r="E59" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F59" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G59" t="s">
         <v>25</v>
       </c>
       <c r="H59" s="1">
-        <v>45712</v>
+        <v>46065</v>
       </c>
       <c r="I59" s="2">
-        <v>8.555092592592592E-4</v>
+        <v>8.4380787037037041E-4</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.45">
@@ -2284,16 +2284,16 @@
         <v>12</v>
       </c>
       <c r="F60" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G60" t="s">
         <v>25</v>
       </c>
       <c r="H60" s="1">
-        <v>45712</v>
+        <v>45844</v>
       </c>
       <c r="I60" s="2">
-        <v>8.5812499999999995E-4</v>
+        <v>8.5418981481481468E-4</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.45">
@@ -2307,10 +2307,10 @@
         <v>18</v>
       </c>
       <c r="D61" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E61" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F61" t="s">
         <v>36</v>
@@ -2322,7 +2322,7 @@
         <v>45712</v>
       </c>
       <c r="I61" s="2">
-        <v>3.7812615740740745E-3</v>
+        <v>8.555092592592592E-4</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.45">
@@ -2336,10 +2336,10 @@
         <v>18</v>
       </c>
       <c r="D62" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E62" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F62" t="s">
         <v>36</v>
@@ -2351,7 +2351,7 @@
         <v>45712</v>
       </c>
       <c r="I62" s="2">
-        <v>3.8320717592592595E-3</v>
+        <v>8.5812499999999995E-4</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.45">
@@ -2365,22 +2365,22 @@
         <v>18</v>
       </c>
       <c r="D63" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="E63" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F63" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G63" t="s">
         <v>25</v>
       </c>
       <c r="H63" s="1">
-        <v>46065</v>
-      </c>
-      <c r="I63">
-        <v>11.948</v>
+        <v>45712</v>
+      </c>
+      <c r="I63" s="2">
+        <v>3.7812615740740745E-3</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.45">
@@ -2394,7 +2394,7 @@
         <v>18</v>
       </c>
       <c r="D64" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="E64" t="s">
         <v>24</v>
@@ -2408,25 +2408,25 @@
       <c r="H64" s="1">
         <v>45712</v>
       </c>
-      <c r="I64">
-        <v>12.577999999999999</v>
+      <c r="I64" s="2">
+        <v>3.8320717592592595E-3</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="B65" t="s">
         <v>9</v>
       </c>
       <c r="C65" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D65" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E65" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F65" t="s">
         <v>35</v>
@@ -2437,37 +2437,37 @@
       <c r="H65" s="1">
         <v>46065</v>
       </c>
-      <c r="I65" s="2">
-        <v>8.9262731481481485E-4</v>
+      <c r="I65">
+        <v>11.948</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="B66" t="s">
         <v>9</v>
       </c>
       <c r="C66" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D66" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E66" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F66" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G66" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="H66" s="1">
-        <v>45700</v>
-      </c>
-      <c r="I66" s="2">
-        <v>9.3041666666666674E-4</v>
+        <v>45712</v>
+      </c>
+      <c r="I66">
+        <v>12.577999999999999</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.45">
@@ -2484,19 +2484,19 @@
         <v>22</v>
       </c>
       <c r="E67" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F67" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G67" t="s">
         <v>25</v>
       </c>
       <c r="H67" s="1">
-        <v>45712</v>
+        <v>46065</v>
       </c>
       <c r="I67" s="2">
-        <v>9.4694444444444448E-4</v>
+        <v>8.9262731481481485E-4</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.45">
@@ -2516,16 +2516,16 @@
         <v>12</v>
       </c>
       <c r="F68" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G68" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="H68" s="1">
-        <v>45712</v>
+        <v>45700</v>
       </c>
       <c r="I68" s="2">
-        <v>9.5013888888888882E-4</v>
+        <v>9.3041666666666674E-4</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.45">
@@ -2542,19 +2542,19 @@
         <v>22</v>
       </c>
       <c r="E69" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F69" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G69" t="s">
         <v>25</v>
       </c>
       <c r="H69" s="1">
-        <v>45844</v>
+        <v>45712</v>
       </c>
       <c r="I69" s="2">
-        <v>9.5561342592592594E-4</v>
+        <v>9.4694444444444448E-4</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.45">
@@ -2565,25 +2565,25 @@
         <v>9</v>
       </c>
       <c r="C70" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="D70" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E70" t="s">
         <v>12</v>
       </c>
       <c r="F70" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G70" t="s">
         <v>25</v>
       </c>
       <c r="H70" s="1">
-        <v>46065</v>
+        <v>45712</v>
       </c>
       <c r="I70" s="2">
-        <v>2.8027430555555557E-3</v>
+        <v>9.5013888888888882E-4</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.45">
@@ -2597,22 +2597,22 @@
         <v>10</v>
       </c>
       <c r="D71" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E71" t="s">
         <v>12</v>
       </c>
       <c r="F71" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G71" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="H71" s="1">
-        <v>45700</v>
+        <v>45844</v>
       </c>
       <c r="I71" s="2">
-        <v>2.8997800925925927E-3</v>
+        <v>9.5561342592592594E-4</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.45">
@@ -2623,7 +2623,7 @@
         <v>9</v>
       </c>
       <c r="C72" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="D72" t="s">
         <v>11</v>
@@ -2632,16 +2632,16 @@
         <v>12</v>
       </c>
       <c r="F72" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G72" t="s">
         <v>25</v>
       </c>
       <c r="H72" s="1">
-        <v>45712</v>
+        <v>46065</v>
       </c>
       <c r="I72" s="2">
-        <v>2.9562499999999997E-3</v>
+        <v>2.8027430555555557E-3</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.45">
@@ -2658,19 +2658,19 @@
         <v>11</v>
       </c>
       <c r="E73" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F73" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G73" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="H73" s="1">
-        <v>45712</v>
+        <v>45700</v>
       </c>
       <c r="I73" s="2">
-        <v>2.9950694444444443E-3</v>
+        <v>2.8997800925925927E-3</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.45">
@@ -2687,19 +2687,19 @@
         <v>11</v>
       </c>
       <c r="E74" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F74" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G74" t="s">
         <v>25</v>
       </c>
       <c r="H74" s="1">
-        <v>45844</v>
+        <v>45712</v>
       </c>
       <c r="I74" s="2">
-        <v>3.055648148148148E-3</v>
+        <v>2.9562499999999997E-3</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.45">
@@ -2710,25 +2710,25 @@
         <v>9</v>
       </c>
       <c r="C75" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="D75" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="E75" t="s">
         <v>24</v>
       </c>
       <c r="F75" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G75" t="s">
         <v>25</v>
       </c>
       <c r="H75" s="1">
-        <v>46065</v>
-      </c>
-      <c r="I75">
-        <v>12.601000000000001</v>
+        <v>45712</v>
+      </c>
+      <c r="I75" s="2">
+        <v>2.9950694444444443E-3</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.45">
@@ -2742,22 +2742,22 @@
         <v>10</v>
       </c>
       <c r="D76" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="E76" t="s">
         <v>24</v>
       </c>
       <c r="F76" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G76" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="H76" s="1">
-        <v>45700</v>
-      </c>
-      <c r="I76">
-        <v>13.316000000000001</v>
+        <v>45844</v>
+      </c>
+      <c r="I76" s="2">
+        <v>3.055648148148148E-3</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.45">
@@ -2768,7 +2768,7 @@
         <v>9</v>
       </c>
       <c r="C77" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="D77" t="s">
         <v>23</v>
@@ -2777,74 +2777,74 @@
         <v>24</v>
       </c>
       <c r="F77" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G77" t="s">
         <v>25</v>
       </c>
       <c r="H77" s="1">
-        <v>45712</v>
+        <v>46065</v>
       </c>
       <c r="I77">
-        <v>13.417</v>
+        <v>12.601000000000001</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B78" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="C78" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D78" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E78" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F78" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="G78" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="H78" s="1">
-        <v>45946</v>
-      </c>
-      <c r="I78" s="2">
-        <v>8.7133101851851857E-4</v>
+        <v>45700</v>
+      </c>
+      <c r="I78">
+        <v>13.316000000000001</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B79" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="C79" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D79" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E79" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F79" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G79" t="s">
         <v>25</v>
       </c>
       <c r="H79" s="1">
-        <v>46065</v>
-      </c>
-      <c r="I79" s="2">
-        <v>8.8388888888888881E-4</v>
+        <v>45712</v>
+      </c>
+      <c r="I79">
+        <v>13.417</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.45">
@@ -2864,16 +2864,16 @@
         <v>12</v>
       </c>
       <c r="F80" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G80" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="H80" s="1">
-        <v>45700</v>
+        <v>45946</v>
       </c>
       <c r="I80" s="2">
-        <v>9.0182870370370373E-4</v>
+        <v>8.7133101851851857E-4</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.45">
@@ -2893,16 +2893,16 @@
         <v>12</v>
       </c>
       <c r="F81" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G81" t="s">
         <v>25</v>
       </c>
       <c r="H81" s="1">
-        <v>45844</v>
+        <v>46065</v>
       </c>
       <c r="I81" s="2">
-        <v>9.2168981481481485E-4</v>
+        <v>8.8388888888888881E-4</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.45">
@@ -2916,22 +2916,22 @@
         <v>18</v>
       </c>
       <c r="D82" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E82" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F82" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="G82" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="H82" s="1">
-        <v>45946</v>
-      </c>
-      <c r="I82">
-        <v>12.33</v>
+        <v>45700</v>
+      </c>
+      <c r="I82" s="2">
+        <v>9.0182870370370373E-4</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.45">
@@ -2945,22 +2945,22 @@
         <v>18</v>
       </c>
       <c r="D83" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E83" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F83" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G83" t="s">
         <v>25</v>
       </c>
       <c r="H83" s="1">
-        <v>46065</v>
-      </c>
-      <c r="I83">
-        <v>12.346</v>
+        <v>45844</v>
+      </c>
+      <c r="I83" s="2">
+        <v>9.2168981481481485E-4</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.45">
@@ -2980,79 +2980,137 @@
         <v>24</v>
       </c>
       <c r="F84" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G84" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="H84" s="1">
-        <v>45700</v>
+        <v>45946</v>
       </c>
       <c r="I84">
-        <v>12.96</v>
+        <v>12.33</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="B85" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C85" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D85" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E85" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F85" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G85" t="s">
         <v>25</v>
       </c>
       <c r="H85" s="1">
-        <v>45844</v>
-      </c>
-      <c r="I85" s="2">
-        <v>8.2354166666666665E-4</v>
+        <v>46065</v>
+      </c>
+      <c r="I85">
+        <v>12.346</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
+        <v>16</v>
+      </c>
+      <c r="B86" t="s">
+        <v>17</v>
+      </c>
+      <c r="C86" t="s">
+        <v>18</v>
+      </c>
+      <c r="D86" t="s">
+        <v>23</v>
+      </c>
+      <c r="E86" t="s">
+        <v>24</v>
+      </c>
+      <c r="F86" t="s">
+        <v>35</v>
+      </c>
+      <c r="G86" t="s">
+        <v>13</v>
+      </c>
+      <c r="H86" s="1">
+        <v>45700</v>
+      </c>
+      <c r="I86">
+        <v>12.96</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A87" t="s">
         <v>37</v>
       </c>
-      <c r="B86" t="s">
-        <v>9</v>
-      </c>
-      <c r="C86" t="s">
+      <c r="B87" t="s">
+        <v>9</v>
+      </c>
+      <c r="C87" t="s">
         <v>19</v>
       </c>
-      <c r="D86" t="s">
+      <c r="D87" t="s">
+        <v>22</v>
+      </c>
+      <c r="E87" t="s">
+        <v>12</v>
+      </c>
+      <c r="F87" t="s">
+        <v>38</v>
+      </c>
+      <c r="G87" t="s">
+        <v>25</v>
+      </c>
+      <c r="H87" s="1">
+        <v>45844</v>
+      </c>
+      <c r="I87" s="2">
+        <v>8.2354166666666665E-4</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A88" t="s">
+        <v>37</v>
+      </c>
+      <c r="B88" t="s">
+        <v>9</v>
+      </c>
+      <c r="C88" t="s">
+        <v>19</v>
+      </c>
+      <c r="D88" t="s">
         <v>11</v>
       </c>
-      <c r="E86" t="s">
-        <v>24</v>
-      </c>
-      <c r="F86" t="s">
+      <c r="E88" t="s">
+        <v>24</v>
+      </c>
+      <c r="F88" t="s">
         <v>38</v>
       </c>
-      <c r="G86" t="s">
-        <v>25</v>
-      </c>
-      <c r="H86" s="1">
+      <c r="G88" t="s">
+        <v>25</v>
+      </c>
+      <c r="H88" s="1">
         <v>45844</v>
       </c>
-      <c r="I86" s="2">
+      <c r="I88" s="2">
         <v>3.201238425925926E-3</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I68" xr:uid="{24732CBF-5850-4CE8-9E62-B42B0032864B}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I86">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I88">
       <sortCondition ref="A1:A68"/>
     </sortState>
   </autoFilter>

</xml_diff>

<commit_message>
updated with NTS results july 2026
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sportnzgroup-my.sharepoint.com/personal/sam_bremer_hpsnz_org_nz/Documents/Desktop/Scripts/Para Tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="882" documentId="13_ncr:1_{1C6954CE-EC5B-43AB-B923-0C939D68B3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54A8AFA1-07A0-492E-BA2C-3CE46966EC24}"/>
+  <xr:revisionPtr revIDLastSave="934" documentId="13_ncr:1_{1C6954CE-EC5B-43AB-B923-0C939D68B3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DEDD849-0FA8-4695-B5A7-091F219EC41D}"/>
   <bookViews>
     <workbookView xWindow="-19298" yWindow="-1837" windowWidth="19396" windowHeight="11475" xr2:uid="{0366F0DF-8659-49CC-A902-2A4788A5E28D}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1942" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2012" uniqueCount="57">
   <si>
     <t>Name</t>
   </si>
@@ -607,7 +607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24732CBF-5850-4CE8-9E62-B42B0032864B}">
-  <dimension ref="A1:N266"/>
+  <dimension ref="A1:N276"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -9120,6 +9120,314 @@
       </c>
       <c r="I266" s="5">
         <v>8.2354166666666665E-4</v>
+      </c>
+    </row>
+    <row r="267" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A267" t="s">
+        <v>32</v>
+      </c>
+      <c r="B267" t="s">
+        <v>16</v>
+      </c>
+      <c r="C267" t="s">
+        <v>14</v>
+      </c>
+      <c r="D267" t="s">
+        <v>43</v>
+      </c>
+      <c r="E267" t="s">
+        <v>23</v>
+      </c>
+      <c r="F267" t="s">
+        <v>37</v>
+      </c>
+      <c r="G267" t="s">
+        <v>24</v>
+      </c>
+      <c r="H267" s="1">
+        <v>46215</v>
+      </c>
+      <c r="I267" s="5">
+        <v>3.5118171296296295E-3</v>
+      </c>
+      <c r="J267">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="268" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A268" t="s">
+        <v>30</v>
+      </c>
+      <c r="B268" t="s">
+        <v>16</v>
+      </c>
+      <c r="C268" t="s">
+        <v>18</v>
+      </c>
+      <c r="D268" t="s">
+        <v>21</v>
+      </c>
+      <c r="E268" t="s">
+        <v>23</v>
+      </c>
+      <c r="F268" t="s">
+        <v>37</v>
+      </c>
+      <c r="G268" t="s">
+        <v>24</v>
+      </c>
+      <c r="H268" s="1">
+        <v>46215</v>
+      </c>
+      <c r="I268" s="5">
+        <v>7.7692129629629639E-4</v>
+      </c>
+      <c r="J268">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="269" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A269" t="s">
+        <v>32</v>
+      </c>
+      <c r="B269" t="s">
+        <v>16</v>
+      </c>
+      <c r="C269" t="s">
+        <v>14</v>
+      </c>
+      <c r="D269" t="s">
+        <v>21</v>
+      </c>
+      <c r="E269" t="s">
+        <v>23</v>
+      </c>
+      <c r="F269" t="s">
+        <v>37</v>
+      </c>
+      <c r="G269" t="s">
+        <v>24</v>
+      </c>
+      <c r="H269" s="1">
+        <v>46214</v>
+      </c>
+      <c r="I269" s="5">
+        <v>8.6296296296296295E-4</v>
+      </c>
+      <c r="J269">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="270" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A270" t="s">
+        <v>45</v>
+      </c>
+      <c r="B270" t="s">
+        <v>16</v>
+      </c>
+      <c r="C270" t="s">
+        <v>17</v>
+      </c>
+      <c r="D270" t="s">
+        <v>21</v>
+      </c>
+      <c r="E270" t="s">
+        <v>23</v>
+      </c>
+      <c r="F270" t="s">
+        <v>37</v>
+      </c>
+      <c r="G270" t="s">
+        <v>24</v>
+      </c>
+      <c r="H270" s="1">
+        <v>46214</v>
+      </c>
+      <c r="I270" s="3">
+        <v>8.7290509259259255E-4</v>
+      </c>
+      <c r="J270">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="271" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A271" t="s">
+        <v>15</v>
+      </c>
+      <c r="B271" t="s">
+        <v>16</v>
+      </c>
+      <c r="C271" t="s">
+        <v>17</v>
+      </c>
+      <c r="D271" t="s">
+        <v>21</v>
+      </c>
+      <c r="E271" t="s">
+        <v>23</v>
+      </c>
+      <c r="F271" t="s">
+        <v>37</v>
+      </c>
+      <c r="G271" t="s">
+        <v>24</v>
+      </c>
+      <c r="H271" s="1">
+        <v>46214</v>
+      </c>
+      <c r="I271" s="3">
+        <v>8.8031250000000002E-4</v>
+      </c>
+      <c r="J271">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="272" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A272" t="s">
+        <v>30</v>
+      </c>
+      <c r="B272" t="s">
+        <v>16</v>
+      </c>
+      <c r="C272" t="s">
+        <v>18</v>
+      </c>
+      <c r="D272" t="s">
+        <v>43</v>
+      </c>
+      <c r="E272" t="s">
+        <v>23</v>
+      </c>
+      <c r="F272" t="s">
+        <v>37</v>
+      </c>
+      <c r="G272" t="s">
+        <v>24</v>
+      </c>
+      <c r="H272" s="1">
+        <v>46214</v>
+      </c>
+      <c r="I272" s="5">
+        <v>3.1974884259259257E-3</v>
+      </c>
+      <c r="J272">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="273" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A273" t="s">
+        <v>27</v>
+      </c>
+      <c r="B273" t="s">
+        <v>9</v>
+      </c>
+      <c r="C273" t="s">
+        <v>10</v>
+      </c>
+      <c r="D273" t="s">
+        <v>22</v>
+      </c>
+      <c r="E273" t="s">
+        <v>23</v>
+      </c>
+      <c r="F273" t="s">
+        <v>37</v>
+      </c>
+      <c r="G273" t="s">
+        <v>24</v>
+      </c>
+      <c r="H273" s="1">
+        <v>46214</v>
+      </c>
+      <c r="I273">
+        <v>11.182</v>
+      </c>
+    </row>
+    <row r="274" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A274" t="s">
+        <v>13</v>
+      </c>
+      <c r="B274" t="s">
+        <v>9</v>
+      </c>
+      <c r="C274" t="s">
+        <v>14</v>
+      </c>
+      <c r="D274" t="s">
+        <v>22</v>
+      </c>
+      <c r="E274" t="s">
+        <v>23</v>
+      </c>
+      <c r="F274" t="s">
+        <v>37</v>
+      </c>
+      <c r="G274" t="s">
+        <v>24</v>
+      </c>
+      <c r="H274" s="1">
+        <v>46214</v>
+      </c>
+      <c r="I274">
+        <v>10.834</v>
+      </c>
+    </row>
+    <row r="275" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A275" t="s">
+        <v>15</v>
+      </c>
+      <c r="B275" t="s">
+        <v>16</v>
+      </c>
+      <c r="C275" t="s">
+        <v>17</v>
+      </c>
+      <c r="D275" t="s">
+        <v>22</v>
+      </c>
+      <c r="E275" t="s">
+        <v>23</v>
+      </c>
+      <c r="F275" t="s">
+        <v>37</v>
+      </c>
+      <c r="G275" t="s">
+        <v>24</v>
+      </c>
+      <c r="H275" s="1">
+        <v>46214</v>
+      </c>
+      <c r="I275">
+        <v>12.356</v>
+      </c>
+    </row>
+    <row r="276" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A276" t="s">
+        <v>32</v>
+      </c>
+      <c r="B276" t="s">
+        <v>16</v>
+      </c>
+      <c r="C276" t="s">
+        <v>14</v>
+      </c>
+      <c r="D276" t="s">
+        <v>21</v>
+      </c>
+      <c r="E276" t="s">
+        <v>23</v>
+      </c>
+      <c r="F276" t="s">
+        <v>37</v>
+      </c>
+      <c r="G276" t="s">
+        <v>24</v>
+      </c>
+      <c r="H276" s="1">
+        <v>46214</v>
+      </c>
+      <c r="I276">
+        <v>12.567</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed file name and added goldmine dta
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sportnzgroup-my.sharepoint.com/personal/sam_bremer_hpsnz_org_nz/Documents/Desktop/Scripts/Para Tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="936" documentId="13_ncr:1_{1C6954CE-EC5B-43AB-B923-0C939D68B3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B510F768-845B-4B48-BB1B-44F4B9E1030A}"/>
+  <xr:revisionPtr revIDLastSave="937" documentId="13_ncr:1_{1C6954CE-EC5B-43AB-B923-0C939D68B3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4A9C892-0488-4027-A2E8-A71EAEE5AF17}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0366F0DF-8659-49CC-A902-2A4788A5E28D}"/>
+    <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11295" xr2:uid="{0366F0DF-8659-49CC-A902-2A4788A5E28D}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -614,7 +614,7 @@
     <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.5703125" customWidth="1"/>
     <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="19.5703125" bestFit="1" customWidth="1"/>

</xml_diff>